<commit_message>
Update MIS_Consolidated.xlsx with latest execution report
</commit_message>
<xml_diff>
--- a/Report Files/MIS_Consolidated.xlsx
+++ b/Report Files/MIS_Consolidated.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="30">
   <si>
     <t>Module</t>
   </si>
@@ -34,8 +34,8 @@
     <t>PO</t>
   </si>
   <si>
-    <t xml:space="preserve">Batches page (second pass) load time: 1.35 sec
-All-transactions page load time: 7.7 sec</t>
+    <t xml:space="preserve">Batches page (second pass) load time: 1.48 sec
+All-transactions page load time: 7.71 sec</t>
   </si>
   <si>
     <t>Header Comparison Result: MATCH (25 columns compared against C:\Users\akspa\OneDrive\Desktop\Automation\MIS-Stagging\sample_excel\sample_po.csv).</t>
@@ -53,7 +53,7 @@
     <t>VCC</t>
   </si>
   <si>
-    <t>All-transactions page load time: 7.59 sec</t>
+    <t>All-transactions page load time: 8.16 sec</t>
   </si>
   <si>
     <t>Header Comparison Result: MATCH (25 columns compared against C:\Users\akspa\OneDrive\Desktop\Automation\MIS-Stagging\sample_excel\sample_vcc.csv).</t>
@@ -65,35 +65,29 @@
     <t>Trial Balance</t>
   </si>
   <si>
-    <t>Trial Balance upload duration: 2 min 1 sec</t>
-  </si>
-  <si>
-    <t>loading Trial Balance time is taking more than 2seconds.</t>
+    <t>Currently, no actions were performed in this module.</t>
   </si>
   <si>
     <t>Payroll</t>
   </si>
   <si>
-    <t>Payroll upload duration: 3.64 sec</t>
+    <t>Payroll upload duration: 4.99 sec</t>
   </si>
   <si>
     <t>Internal Accounts</t>
   </si>
   <si>
-    <t>Import duration: 1.06 sec</t>
+    <t>Import duration: 1.07 sec</t>
   </si>
   <si>
     <t>Trial Balance Revisit</t>
   </si>
   <si>
-    <t>Currently, no actions were performed in this module.</t>
-  </si>
-  <si>
     <t>Budget</t>
   </si>
   <si>
     <t xml:space="preserve">All dropdown became clickable in: 0 sec
-Budget CSV upload duration: 1.87 sec</t>
+Budget CSV upload duration: 1.85 sec</t>
   </si>
   <si>
     <t>Financial Year</t>
@@ -102,12 +96,13 @@
     <t>Reports</t>
   </si>
   <si>
-    <t xml:space="preserve">All Vendor Transactions page load time: 10.3 sec
-All Vendor Transactions CSV download duration: 5.72 sec
-Balance Sheet page load time: 1.54 sec</t>
-  </si>
-  <si>
-    <t>All Vendor Transactions loading is taking more than 2 seconds.</t>
+    <t xml:space="preserve">All Vendor Transactions page load time: 8.5 sec
+All Vendor Transactions CSV download duration: 8.99 sec
+Balance Sheet page load time: 3.05 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Vendor Transactions loading is taking more than 2 seconds.
+Balance Sheet loading is taking more than 2 seconds.</t>
   </si>
   <si>
     <t>Audit Logs</t>
@@ -571,27 +566,27 @@
         <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
@@ -608,10 +603,10 @@
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -628,7 +623,7 @@
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>11</v>
@@ -643,15 +638,15 @@
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
@@ -668,7 +663,7 @@
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>11</v>
@@ -683,24 +678,24 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>11</v>
@@ -708,7 +703,7 @@
     </row>
     <row r="11" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
@@ -723,7 +718,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>